<commit_message>
Revise CrewPay workbook proof controls
</commit_message>
<xml_diff>
--- a/CrewPay_Ledger_Workbook.xlsx
+++ b/CrewPay_Ledger_Workbook.xlsx
@@ -22,7 +22,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar Sync Log" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dropdown Lists" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Worker Proof'!$1:$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'Worker Proof'!$A$1:$M$34</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -202,7 +205,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -214,6 +217,20 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FCE7E7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E5E7EB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F8D7DA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -579,7 +596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -723,14 +740,29 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Manual-first rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>The workbook must remain usable manually. Any future script helper should write back to the Proof Exports, Access Log, Correction Log, or Calendar Sync Log tabs instead of becoming the source of truth.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A28:F28"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A31:F31"/>
     <mergeCell ref="A22:F22"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="A7:F7"/>
@@ -845,10 +877,8 @@
           <t>P-4003</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
+      <c r="F2" s="12" t="n">
+        <v>46181</v>
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
@@ -877,6 +907,17 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>'Time Entries'!$A$2:$A$200</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>Workers!$A$2:$A$200</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>'Pay Periods'!$A$2:$A$100</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -986,20 +1027,14 @@
           <t>Maya Ellis</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-      <c r="G2" s="11" t="inlineStr">
-        <is>
-          <t>08:00</t>
-        </is>
-      </c>
-      <c r="H2" s="11" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
+      <c r="F2" s="12" t="n">
+        <v>46184</v>
+      </c>
+      <c r="G2" s="14" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="H2" s="14" t="n">
+        <v>0.6666666666666666</v>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
@@ -1043,20 +1078,14 @@
           <t>Leo Grant</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="G3" s="11" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="H3" s="11" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
+      <c r="F3" s="12" t="n">
+        <v>46185</v>
+      </c>
+      <c r="G3" s="14" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="H3" s="14" t="n">
+        <v>0.5416666666666666</v>
       </c>
       <c r="I3" s="11" t="inlineStr">
         <is>
@@ -1071,7 +1100,13 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>Jobs!$A$2:$A$200</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>Workers!$A$2:$A$200</formula1>
+    </dataValidation>
     <dataValidation sqref="I2:I100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
       <formula1>'Dropdown Lists'!$G$2:$G$5</formula1>
     </dataValidation>
@@ -1177,10 +1212,8 @@
           <t>N-9001</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
-        <is>
-          <t>2026-06-08 12:15</t>
-        </is>
+      <c r="B2" s="16" t="n">
+        <v>46181.51041666666</v>
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
@@ -1227,10 +1260,8 @@
           <t>Posted</t>
         </is>
       </c>
-      <c r="L2" s="11" t="inlineStr">
-        <is>
-          <t>2026-06-08 12:15</t>
-        </is>
+      <c r="L2" s="16" t="n">
+        <v>46181.51041666666</v>
       </c>
       <c r="M2" s="11" t="inlineStr">
         <is>
@@ -1244,10 +1275,8 @@
           <t>N-9002</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
-        <is>
-          <t>2026-06-09 08:20</t>
-        </is>
+      <c r="B3" s="16" t="n">
+        <v>46182.34722222222</v>
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
@@ -1282,7 +1311,7 @@
           <t>Draft</t>
         </is>
       </c>
-      <c r="L3" s="11" t="inlineStr"/>
+      <c r="L3" s="16" t="n"/>
       <c r="M3" s="11" t="inlineStr">
         <is>
           <t>Email-ready text only; no send automation.</t>
@@ -1290,9 +1319,15 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="5">
     <dataValidation sqref="D2:D100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
       <formula1>'Dropdown Lists'!$H$2:$H$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>Workers!$A$2:$A$200</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>'Pay Periods'!$A$2:$A$100</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
       <formula1>'Dropdown Lists'!$I$2:$I$4</formula1>
@@ -1409,17 +1444,15 @@
           <t>cal-demo-oak-001</t>
         </is>
       </c>
-      <c r="G2" s="11" t="inlineStr">
-        <is>
-          <t>2026-06-11</t>
-        </is>
+      <c r="G2" s="12" t="n">
+        <v>46184</v>
       </c>
       <c r="H2" s="11" t="inlineStr">
         <is>
           <t>Not Synced</t>
         </is>
       </c>
-      <c r="I2" s="11" t="inlineStr"/>
+      <c r="I2" s="16" t="n"/>
       <c r="J2" s="11" t="inlineStr">
         <is>
           <t>Calendar is reference only, not proof.</t>
@@ -1427,7 +1460,13 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>Jobs!$A$2:$A$200</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>Workers!$A$2:$A$200</formula1>
+    </dataValidation>
     <dataValidation sqref="H2:H100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
       <formula1>'Dropdown Lists'!$K$2:$K$5</formula1>
     </dataValidation>
@@ -9175,10 +9214,19 @@
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>$S2&lt;&gt;""</formula>
     </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>IFERROR(VLOOKUP($B2,Workers!$A:$E,5,FALSE)="Inactive",FALSE)</formula>
+    </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="3">
     <dataValidation sqref="P2:P200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
       <formula1>'Dropdown Lists'!$C$2:$C$7</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>Workers!$A$2:$A$200</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>Jobs!$A$2:$A$200</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12357,12 +12405,15 @@
       <formula>AND($F2="Finalized",$G2="Unpaid")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="F2:F100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
       <formula1>'Dropdown Lists'!$D$2:$D$4</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
       <formula1>'Dropdown Lists'!$E$2:$E$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>Workers!$A$2:$A$200</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12373,7 +12424,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -12484,6 +12535,17 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>Proof Selector Check</t>
+        </is>
+      </c>
+      <c r="B10" s="11">
+        <f>IFERROR(IF(VLOOKUP($B$4,'Pay Periods'!$A:$O,2,FALSE)=$B$3,"OK - worker/pay period match","CHECK SELECTION - pay period belongs to another worker"),"CHECK SELECTION")</f>
+        <v/>
+      </c>
+    </row>
     <row r="12">
       <c r="A12" s="24" t="inlineStr">
         <is>
@@ -12553,7 +12615,7 @@
     </row>
     <row r="13">
       <c r="A13">
-        <f>FILTER({'Time Entries'!A2:A200,'Time Entries'!F2:F200,'Time Entries'!D2:D200,'Time Entries'!E2:E200,'Time Entries'!J2:J200,'Time Entries'!K2:K200,'Time Entries'!L2:L200,'Time Entries'!M2:M200,'Time Entries'!N2:N200,'Time Entries'!O2:O200,'Time Entries'!P2:P200,'Time Entries'!S2:S200,'Time Entries'!T2:T200},'Time Entries'!B2:B200=$B$3,'Time Entries'!F2:F200&gt;=VLOOKUP($B$4,'Pay Periods'!$A:$O,4,FALSE),'Time Entries'!F2:F200&lt;=VLOOKUP($B$4,'Pay Periods'!$A:$O,5,FALSE))</f>
+        <f>IF($B$10&lt;&gt;"OK - worker/pay period match","Check selected worker/pay period before printing proof",FILTER({'Time Entries'!A2:A200,'Time Entries'!F2:F200,'Time Entries'!D2:D200,'Time Entries'!E2:E200,'Time Entries'!J2:J200,'Time Entries'!K2:K200,'Time Entries'!L2:L200,'Time Entries'!M2:M200,'Time Entries'!N2:N200,'Time Entries'!O2:O200,'Time Entries'!P2:P200,'Time Entries'!S2:S200,'Time Entries'!T2:T200},'Time Entries'!B2:B200=$B$3,'Time Entries'!F2:F200&gt;=VLOOKUP($B$4,'Pay Periods'!$A:$O,4,FALSE),'Time Entries'!F2:F200&lt;=VLOOKUP($B$4,'Pay Periods'!$A:$O,5,FALSE)))</f>
         <v/>
       </c>
     </row>
@@ -12564,7 +12626,7 @@
         </is>
       </c>
       <c r="B30" s="19">
-        <f>IFERROR(VLOOKUP($B$4,'Pay Periods'!$A:$O,8,FALSE),0)</f>
+        <f>IF($B$10&lt;&gt;"OK - worker/pay period match",0,SUMIFS('Time Entries'!$J:$J,'Time Entries'!$B:$B,$B$3,'Time Entries'!$F:$F,"&gt;="&amp;VLOOKUP($B$4,'Pay Periods'!$A:$O,4,FALSE),'Time Entries'!$F:$F,"&lt;="&amp;VLOOKUP($B$4,'Pay Periods'!$A:$O,5,FALSE),'Time Entries'!$P:$P,"&lt;&gt;Draft",'Time Entries'!$P:$P,"&lt;&gt;Rejected"))</f>
         <v/>
       </c>
     </row>
@@ -12575,7 +12637,7 @@
         </is>
       </c>
       <c r="B31" s="20">
-        <f>IFERROR(VLOOKUP($B$4,'Pay Periods'!$A:$O,9,FALSE),0)</f>
+        <f>IF($B$10&lt;&gt;"OK - worker/pay period match",0,SUMIFS('Time Entries'!$L:$L,'Time Entries'!$B:$B,$B$3,'Time Entries'!$F:$F,"&gt;="&amp;VLOOKUP($B$4,'Pay Periods'!$A:$O,4,FALSE),'Time Entries'!$F:$F,"&lt;="&amp;VLOOKUP($B$4,'Pay Periods'!$A:$O,5,FALSE),'Time Entries'!$P:$P,"&lt;&gt;Draft",'Time Entries'!$P:$P,"&lt;&gt;Rejected"))</f>
         <v/>
       </c>
     </row>
@@ -12586,7 +12648,7 @@
         </is>
       </c>
       <c r="B32" s="20">
-        <f>IFERROR(VLOOKUP($B$4,'Pay Periods'!$A:$O,10,FALSE),0)</f>
+        <f>IF($B$10&lt;&gt;"OK - worker/pay period match",0,SUMIFS('Time Entries'!$M:$M,'Time Entries'!$B:$B,$B$3,'Time Entries'!$F:$F,"&gt;="&amp;VLOOKUP($B$4,'Pay Periods'!$A:$O,4,FALSE),'Time Entries'!$F:$F,"&lt;="&amp;VLOOKUP($B$4,'Pay Periods'!$A:$O,5,FALSE),'Time Entries'!$P:$P,"&lt;&gt;Draft",'Time Entries'!$P:$P,"&lt;&gt;Rejected"))</f>
         <v/>
       </c>
     </row>
@@ -12597,7 +12659,7 @@
         </is>
       </c>
       <c r="B33" s="20">
-        <f>IFERROR(VLOOKUP($B$4,'Pay Periods'!$A:$O,11,FALSE),0)</f>
+        <f>IF($B$10&lt;&gt;"OK - worker/pay period match",0,SUMIFS('Time Entries'!$N:$N,'Time Entries'!$B:$B,$B$3,'Time Entries'!$F:$F,"&gt;="&amp;VLOOKUP($B$4,'Pay Periods'!$A:$O,4,FALSE),'Time Entries'!$F:$F,"&lt;="&amp;VLOOKUP($B$4,'Pay Periods'!$A:$O,5,FALSE),'Time Entries'!$P:$P,"&lt;&gt;Draft",'Time Entries'!$P:$P,"&lt;&gt;Rejected"))</f>
         <v/>
       </c>
     </row>
@@ -12608,7 +12670,7 @@
         </is>
       </c>
       <c r="B34" s="20">
-        <f>IFERROR(VLOOKUP($B$4,'Pay Periods'!$A:$O,12,FALSE),0)</f>
+        <f>B31+B32-B33</f>
         <v/>
       </c>
     </row>
@@ -12617,6 +12679,11 @@
     <mergeCell ref="D3:H6"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <conditionalFormatting sqref="A10:B10">
+    <cfRule type="expression" priority="1" dxfId="3">
+      <formula>$B$10&lt;&gt;"OK - worker/pay period match"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
       <formula1>'Dropdown Lists'!$E$2:$E$3</formula1>
@@ -12629,6 +12696,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -12725,10 +12793,8 @@
           <t>Print</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
-        <is>
-          <t>2026-06-08 12:05</t>
-        </is>
+      <c r="F2" s="16" t="n">
+        <v>46181.50347222222</v>
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
@@ -12772,10 +12838,8 @@
           <t>CSV</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
-        <is>
-          <t>2026-06-09 09:30</t>
-        </is>
+      <c r="F3" s="16" t="n">
+        <v>46182.39583333334</v>
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
@@ -12794,7 +12858,13 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="3">
+    <dataValidation sqref="B2:B100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>Workers!$A$2:$A$200</formula1>
+    </dataValidation>
+    <dataValidation sqref="D2:D100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>'Pay Periods'!$A$2:$A$100</formula1>
+    </dataValidation>
     <dataValidation sqref="E2:E100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
       <formula1>'Dropdown Lists'!$F$2:$F$4</formula1>
     </dataValidation>
@@ -12890,10 +12960,8 @@
           <t>Inactive</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
-        <is>
-          <t>2026-06-09 08:00</t>
-        </is>
+      <c r="F2" s="16" t="n">
+        <v>46182.33333333334</v>
       </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
@@ -12907,7 +12975,10 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="B2:B100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from the approved workbook range." type="list">
+      <formula1>Workers!$A$2:$A$200</formula1>
+    </dataValidation>
     <dataValidation sqref="D2:E100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
       <formula1>'Dropdown Lists'!$A$2:$A$3</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
Add workbook bridge intake tabs
</commit_message>
<xml_diff>
--- a/CrewPay_Ledger_Workbook.xlsx
+++ b/CrewPay_Ledger_Workbook.xlsx
@@ -22,7 +22,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Admin Notices" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendar Sync Log" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dropdown Lists" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Config" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending Worker Intake" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending Pay Period Intake" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending Time Entries" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="App Submission Log" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bridge Schema" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dropdown Lists" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Workers'!$A$1:$H$4</definedName>
@@ -37,6 +43,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Schedule'!$A$1:$K$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Admin Notices'!$A$1:$M$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Calendar Sync Log'!$A$1:$J$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'App Config'!$A$1:$C$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Pending Worker Intake'!$A$1:$M$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Pending Pay Period Intake'!$A$1:$N$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Pending Time Entries'!$A$1:$Q$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'App Submission Log'!$A$1:$K$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Bridge Schema'!$A$1:$G$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2403,313 +2415,848 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>Access Status</t>
+          <t>Config Key</t>
         </is>
       </c>
       <c r="B1" s="12" t="inlineStr">
         <is>
-          <t>Job Status</t>
+          <t>Config Value</t>
         </is>
       </c>
       <c r="C1" s="12" t="inlineStr">
         <is>
-          <t>Approval Status</t>
-        </is>
-      </c>
-      <c r="D1" s="12" t="inlineStr">
-        <is>
-          <t>Pay Period Status</t>
-        </is>
-      </c>
-      <c r="E1" s="12" t="inlineStr">
-        <is>
-          <t>Payment Status</t>
-        </is>
-      </c>
-      <c r="F1" s="12" t="inlineStr">
-        <is>
-          <t>Export Type</t>
-        </is>
-      </c>
-      <c r="G1" s="12" t="inlineStr">
-        <is>
-          <t>Schedule Status</t>
-        </is>
-      </c>
-      <c r="H1" s="12" t="inlineStr">
-        <is>
-          <t>Recipient Type</t>
-        </is>
-      </c>
-      <c r="I1" s="12" t="inlineStr">
-        <is>
-          <t>Delivery Method</t>
-        </is>
-      </c>
-      <c r="J1" s="12" t="inlineStr">
-        <is>
-          <t>Notice Status</t>
-        </is>
-      </c>
-      <c r="K1" s="12" t="inlineStr">
-        <is>
-          <t>Sync Status</t>
-        </is>
-      </c>
-      <c r="M1" s="50" t="inlineStr">
-        <is>
-          <t>Demo Config</t>
-        </is>
-      </c>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="E1" s="9" t="inlineStr">
+        <is>
+          <t>Bridge boundary</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="n"/>
+      <c r="G1" s="10" t="n"/>
+      <c r="H1" s="10" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Workbook Source Of Truth</t>
         </is>
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>TRUE</t>
         </is>
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="D2" s="14" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E2" s="14" t="inlineStr">
-        <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="F2" s="14" t="inlineStr">
-        <is>
-          <t>Print</t>
-        </is>
-      </c>
-      <c r="G2" s="14" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="H2" s="14" t="inlineStr">
-        <is>
-          <t>Worker</t>
-        </is>
-      </c>
-      <c r="I2" s="14" t="inlineStr">
-        <is>
-          <t>Workbook</t>
-        </is>
-      </c>
-      <c r="J2" s="14" t="inlineStr">
-        <is>
-          <t>Draft</t>
-        </is>
-      </c>
-      <c r="K2" s="14" t="inlineStr">
-        <is>
-          <t>Not Synced</t>
-        </is>
-      </c>
-      <c r="M2" s="51" t="inlineStr">
-        <is>
-          <t>Support/config tab for demo dropdowns. Not part of the public workflow.</t>
-        </is>
-      </c>
+          <t>Workbook remains final authority.</t>
+        </is>
+      </c>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>The workbook remains source of truth. The app may submit controlled intake records through Apps Script after deployment.</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="n"/>
+      <c r="G2" s="10" t="n"/>
+      <c r="H2" s="10" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>Inactive</t>
+          <t>App Role</t>
         </is>
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Paused</t>
+          <t>Companion Input Layer</t>
         </is>
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>Submitted</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>Finalized</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="F3" s="13" t="inlineStr">
-        <is>
-          <t>PDF</t>
-        </is>
-      </c>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>Scheduled</t>
-        </is>
-      </c>
-      <c r="H3" s="13" t="inlineStr">
-        <is>
-          <t>All Active Workers</t>
-        </is>
-      </c>
-      <c r="I3" s="13" t="inlineStr">
-        <is>
-          <t>Email Ready</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="inlineStr">
-        <is>
-          <t>Posted</t>
-        </is>
-      </c>
-      <c r="K3" s="13" t="inlineStr">
-        <is>
-          <t>Synced</t>
-        </is>
-      </c>
+          <t>App submits controlled intake records only.</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="n"/>
+      <c r="F3" s="10" t="n"/>
+      <c r="G3" s="10" t="n"/>
+      <c r="H3" s="10" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="n"/>
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>Backend Type</t>
+        </is>
+      </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Google Apps Script Web App</t>
         </is>
       </c>
       <c r="C4" s="14" t="inlineStr">
         <is>
-          <t>Approved</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="n"/>
-      <c r="F4" s="14" t="inlineStr">
-        <is>
-          <t>CSV</t>
-        </is>
-      </c>
-      <c r="G4" s="14" t="inlineStr">
-        <is>
-          <t>Completed</t>
-        </is>
-      </c>
-      <c r="H4" s="14" t="n"/>
-      <c r="I4" s="14" t="inlineStr">
-        <is>
-          <t>Gmail Sent</t>
-        </is>
-      </c>
-      <c r="J4" s="14" t="inlineStr">
-        <is>
-          <t>Sent</t>
-        </is>
-      </c>
-      <c r="K4" s="14" t="inlineStr">
-        <is>
-          <t>Failed</t>
-        </is>
-      </c>
+          <t>No separate backend server/database.</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="n"/>
+      <c r="F4" s="10" t="n"/>
+      <c r="G4" s="10" t="n"/>
+      <c r="H4" s="10" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="n"/>
-      <c r="B5" s="13" t="n"/>
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Endpoint URL</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>PASTE_DEPLOYED_APPS_SCRIPT_WEB_APP_URL_HERE</t>
+        </is>
+      </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Finalized</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="n"/>
-      <c r="E5" s="13" t="n"/>
-      <c r="F5" s="13" t="n"/>
-      <c r="G5" s="13" t="inlineStr">
-        <is>
-          <t>Canceled</t>
-        </is>
-      </c>
-      <c r="H5" s="13" t="n"/>
-      <c r="I5" s="13" t="n"/>
-      <c r="J5" s="13" t="inlineStr">
-        <is>
-          <t>Archived</t>
-        </is>
-      </c>
-      <c r="K5" s="13" t="inlineStr">
-        <is>
-          <t>Skipped</t>
+          <t>Set after Apps Script deployment.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="n"/>
-      <c r="B6" s="14" t="n"/>
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Bridge Enabled</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="n"/>
-      <c r="E6" s="14" t="n"/>
-      <c r="F6" s="14" t="n"/>
-      <c r="G6" s="14" t="n"/>
-      <c r="H6" s="14" t="n"/>
-      <c r="I6" s="14" t="n"/>
-      <c r="J6" s="14" t="n"/>
-      <c r="K6" s="14" t="n"/>
+          <t>Turn TRUE only after deployment/testing.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="n"/>
-      <c r="B7" s="13" t="n"/>
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Shared Token Required</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Rejected</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="n"/>
-      <c r="E7" s="13" t="n"/>
-      <c r="F7" s="13" t="n"/>
-      <c r="G7" s="13" t="n"/>
-      <c r="H7" s="13" t="n"/>
-      <c r="I7" s="13" t="n"/>
-      <c r="J7" s="13" t="n"/>
-      <c r="K7" s="13" t="n"/>
+          <t>Browser-visible token is not full security; use private/demo boundary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Intake Review Required</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>App submissions should be reviewed before final record use.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C8"/>
+  <mergeCells count="2">
+    <mergeCell ref="E2:H4"/>
+    <mergeCell ref="E1:H1"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
+      <formula1>'Dropdown Lists'!$M$2:$M$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="B6:B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
+      <formula1>'Dropdown Lists'!$M$2:$M$3</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Intake ID</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Submitted At</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Submission Source</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>Submission Status</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>Worker ID</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>Worker Name</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>Access Status</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>Role / Trade</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="J1" s="12" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="K1" s="12" t="inlineStr">
+        <is>
+          <t>Reviewed At</t>
+        </is>
+      </c>
+      <c r="L1" s="12" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="M1" s="12" t="inlineStr">
+        <is>
+          <t>Review Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>PW-0001</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="n">
+        <v>46183.375</v>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>App Demo</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>W-001</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Sample Worker</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>Crew</t>
+        </is>
+      </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>sample@example.com</t>
+        </is>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>Sample pending worker intake row.</t>
+        </is>
+      </c>
+      <c r="K2" s="14" t="inlineStr"/>
+      <c r="L2" s="14" t="inlineStr"/>
+      <c r="M2" s="14" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M2"/>
+  <conditionalFormatting sqref="A2:M200">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$D2="Active"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>$D2="Approved"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>$D2="Paid"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>$D2="Submitted"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$D2="Draft"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="2">
+      <formula>$D2="Finalized"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="2">
+      <formula>$D2="Posted"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="1">
+      <formula>$D2="Email Ready"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="1">
+      <formula>$D2="Scheduled"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="2">
+      <formula>$D2="Planned"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="3">
+      <formula>$D2="Rejected"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="4">
+      <formula>$D2="Inactive"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" dxfId="4">
+      <formula>$D2="Archived"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="4">
+      <formula>$D2="Closed"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="4">
+      <formula>$D2="Canceled"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="4">
+      <formula>$D2="Cancelled"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
+      <formula1>'Dropdown Lists'!$L$2:$L$5</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
+      <formula1>'Dropdown Lists'!$A$2:$A$3</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Intake ID</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Submitted At</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Submission Source</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>Submission Status</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>Pay Period ID</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>Worker ID</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>Worker Name</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>Period Start</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>Period End</t>
+        </is>
+      </c>
+      <c r="J1" s="12" t="inlineStr">
+        <is>
+          <t>Pay Date</t>
+        </is>
+      </c>
+      <c r="K1" s="12" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="L1" s="12" t="inlineStr">
+        <is>
+          <t>Reviewed At</t>
+        </is>
+      </c>
+      <c r="M1" s="12" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="N1" s="12" t="inlineStr">
+        <is>
+          <t>Review Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>PP-0001</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="n">
+        <v>46183.37847222222</v>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>App Demo</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>PP-001</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>W-001</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>Sample Worker</t>
+        </is>
+      </c>
+      <c r="H2" s="15" t="n">
+        <v>46174</v>
+      </c>
+      <c r="I2" s="15" t="n">
+        <v>46180</v>
+      </c>
+      <c r="J2" s="15" t="n">
+        <v>46187</v>
+      </c>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>Sample pending pay period row.</t>
+        </is>
+      </c>
+      <c r="L2" s="14" t="inlineStr"/>
+      <c r="M2" s="14" t="inlineStr"/>
+      <c r="N2" s="14" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N2"/>
+  <conditionalFormatting sqref="A2:N200">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$D2="Active"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>$D2="Approved"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>$D2="Paid"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>$D2="Submitted"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$D2="Draft"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="2">
+      <formula>$D2="Finalized"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="2">
+      <formula>$D2="Posted"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="1">
+      <formula>$D2="Email Ready"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="1">
+      <formula>$D2="Scheduled"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="2">
+      <formula>$D2="Planned"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="3">
+      <formula>$D2="Rejected"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="4">
+      <formula>$D2="Inactive"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" dxfId="4">
+      <formula>$D2="Archived"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="4">
+      <formula>$D2="Closed"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="4">
+      <formula>$D2="Canceled"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="4">
+      <formula>$D2="Cancelled"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
+      <formula1>'Dropdown Lists'!$L$2:$L$5</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="36" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Intake ID</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Submitted At</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Submission Source</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>Submission Status</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>Entry ID</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>Worker ID</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>Worker Name</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>Pay Period ID</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>Work Date</t>
+        </is>
+      </c>
+      <c r="J1" s="12" t="inlineStr">
+        <is>
+          <t>Job / Work Type</t>
+        </is>
+      </c>
+      <c r="K1" s="12" t="inlineStr">
+        <is>
+          <t>Hours</t>
+        </is>
+      </c>
+      <c r="L1" s="12" t="inlineStr">
+        <is>
+          <t>Rate</t>
+        </is>
+      </c>
+      <c r="M1" s="12" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="N1" s="12" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="O1" s="12" t="inlineStr">
+        <is>
+          <t>Reviewed At</t>
+        </is>
+      </c>
+      <c r="P1" s="12" t="inlineStr">
+        <is>
+          <t>Reviewed By</t>
+        </is>
+      </c>
+      <c r="Q1" s="12" t="inlineStr">
+        <is>
+          <t>Review Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>PT-0001</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="n">
+        <v>46183.38194444445</v>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>App Demo</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>E-001</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>W-001</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>Sample Worker</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>PP-001</t>
+        </is>
+      </c>
+      <c r="I2" s="15" t="n">
+        <v>46176</v>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>Sample Work</t>
+        </is>
+      </c>
+      <c r="K2" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="L2" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="M2" s="17">
+        <f>K2*L2</f>
+        <v/>
+      </c>
+      <c r="N2" s="14" t="inlineStr">
+        <is>
+          <t>Sample pending time entry row.</t>
+        </is>
+      </c>
+      <c r="O2" s="14" t="inlineStr"/>
+      <c r="P2" s="14" t="inlineStr"/>
+      <c r="Q2" s="14" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Q2"/>
+  <conditionalFormatting sqref="A2:Q200">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$D2="Active"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>$D2="Approved"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>$D2="Paid"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>$D2="Submitted"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="2">
+      <formula>$D2="Draft"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="6" dxfId="2">
+      <formula>$D2="Finalized"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="7" dxfId="2">
+      <formula>$D2="Posted"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="8" dxfId="1">
+      <formula>$D2="Email Ready"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" dxfId="1">
+      <formula>$D2="Scheduled"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" dxfId="2">
+      <formula>$D2="Planned"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" dxfId="3">
+      <formula>$D2="Rejected"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" dxfId="4">
+      <formula>$D2="Inactive"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="13" dxfId="4">
+      <formula>$D2="Archived"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="14" dxfId="4">
+      <formula>$D2="Closed"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="15" dxfId="4">
+      <formula>$D2="Canceled"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="16" dxfId="4">
+      <formula>$D2="Cancelled"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid value" error="Choose a value from Dropdown Lists." type="list">
+      <formula1>'Dropdown Lists'!$L$2:$L$5</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3013,6 +3560,893 @@
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="G9:H9"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Log ID</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Submitted At</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>Submission Source</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>Related Intake ID</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>Related Worker ID</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>Related Pay Period ID</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+      <c r="J1" s="12" t="inlineStr">
+        <is>
+          <t>Raw Payload Summary</t>
+        </is>
+      </c>
+      <c r="K1" s="12" t="inlineStr">
+        <is>
+          <t>Handled By Script Version</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>AL-0001</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="n">
+        <v>46183.38541666666</v>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>healthCheck</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>App Demo</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr"/>
+      <c r="G2" s="14" t="inlineStr"/>
+      <c r="H2" s="14" t="inlineStr"/>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>Sample app submission log row.</t>
+        </is>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>Sample only.</t>
+        </is>
+      </c>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>Not deployed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Target Tab</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Required Fields</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>Optional Fields</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>Success Response</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>Error Conditions</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>healthCheck</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>App Submission Log</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>client_version, submission_source</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>{ok:true, action:"healthCheck", workbook:"CrewPay Ledger"}</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Bridge disabled; workbook unavailable</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>Readiness check only; may log a health check row if desired.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>getWorkbookSchema</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Bridge Schema / Dropdown Lists</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>schema_version</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>{ok:true, config:{...}, dropdowns:{...}}</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Bridge disabled; schema unavailable</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>Return allowed tabs, writable fields, and dropdown values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>submitWorkerIntake</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Pending Worker Intake</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>worker_name, access_status, role_trade, contact</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>worker_id, notes, idempotency_key</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>{ok:true, intake_id:'PW-####'}</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Missing required field; duplicate submission; invalid access status</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>First landing zone for worker records from the app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>submitPayPeriod</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Pending Pay Period Intake</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>pay_period_id, worker_id, period_start, period_end</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>worker_name, pay_date, notes, idempotency_key</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>{ok:true, intake_id:'PP-####'}</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>Invalid date range; missing worker; duplicate submission</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>Pending setup only. Final Pay Periods tab remains workbook/admin reviewed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>submitTimeEntry</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Pending Time Entries</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>worker_id, pay_period_id, work_date, job_work_type, hours, rate</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>worker_name, entry_id, notes, idempotency_key</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>{ok:true, intake_id:'PT-####'}</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Inactive worker; invalid hours/rate; duplicate submission</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>Safest first write target for app time entries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>logProofExport</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Proof Exports</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>worker_id, pay_period_id, export_type, export_reference</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>worker_name, notes</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>{ok:true, export_id:'X-####'}</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Worker/pay period mismatch; invalid export type</t>
+        </is>
+      </c>
+      <c r="G7" s="13" t="inlineStr">
+        <is>
+          <t>Do not write Worker Proof directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>logCorrection</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Correction Log</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>entry_id, worker_id, pay_period_id, correction_reason, original_value_summary, new_value_summary</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>worker_name, notes</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>{ok:true, correction_id:'C-####'}</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>Missing proof context; duplicate correction</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>Corrections must be visible, not silent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>logAccessChange</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Access Log</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>worker_id, previous_status, new_status, reason</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>worker_name</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>{ok:true, log_id:'A-####'}</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Invalid status; missing reason</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>Future access changes must preserve historical proof.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>createAdminNotice</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Admin Notices</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>recipient_type, subject, message</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>worker_id, worker_name, related_pay_period_id, notes</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>{ok:true, notice_id:'N-####'}</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>Invalid recipient type; missing message</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>Creates a one-way notice row only; sending is separate.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Access Status</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Job Status</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Approval Status</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>Pay Period Status</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>Payment Status</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>Export Type</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>Schedule Status</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>Recipient Type</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>Delivery Method</t>
+        </is>
+      </c>
+      <c r="J1" s="12" t="inlineStr">
+        <is>
+          <t>Notice Status</t>
+        </is>
+      </c>
+      <c r="K1" s="12" t="inlineStr">
+        <is>
+          <t>Sync Status</t>
+        </is>
+      </c>
+      <c r="L1" s="12" t="inlineStr">
+        <is>
+          <t>Submission Status</t>
+        </is>
+      </c>
+      <c r="M1" s="12" t="inlineStr">
+        <is>
+          <t>Boolean Flag</t>
+        </is>
+      </c>
+      <c r="O1" s="50" t="inlineStr">
+        <is>
+          <t>Demo Config</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>Unpaid</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Print</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>Worker</t>
+        </is>
+      </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>Workbook</t>
+        </is>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>Not Synced</t>
+        </is>
+      </c>
+      <c r="L2" s="14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="M2" s="14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="O2" s="51" t="inlineStr">
+        <is>
+          <t>Support/config tab for demo dropdowns. Not part of the public workflow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Inactive</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Paused</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Submitted</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Finalized</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>All Active Workers</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>Email Ready</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>Posted</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>Synced</t>
+        </is>
+      </c>
+      <c r="L3" s="13" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="M3" s="13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="n"/>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="n"/>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>CSV</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="n"/>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>Gmail Sent</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="L4" s="14" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="M4" s="14" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="n"/>
+      <c r="B5" s="13" t="n"/>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Finalized</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="n"/>
+      <c r="E5" s="13" t="n"/>
+      <c r="F5" s="13" t="n"/>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>Canceled</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="n"/>
+      <c r="I5" s="13" t="n"/>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>Archived</t>
+        </is>
+      </c>
+      <c r="K5" s="13" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="M5" s="13" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="n"/>
+      <c r="B6" s="14" t="n"/>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="n"/>
+      <c r="E6" s="14" t="n"/>
+      <c r="F6" s="14" t="n"/>
+      <c r="G6" s="14" t="n"/>
+      <c r="H6" s="14" t="n"/>
+      <c r="I6" s="14" t="n"/>
+      <c r="J6" s="14" t="n"/>
+      <c r="K6" s="14" t="n"/>
+      <c r="L6" s="14" t="n"/>
+      <c r="M6" s="14" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="n"/>
+      <c r="B7" s="13" t="n"/>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Rejected</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="n"/>
+      <c r="E7" s="13" t="n"/>
+      <c r="F7" s="13" t="n"/>
+      <c r="G7" s="13" t="n"/>
+      <c r="H7" s="13" t="n"/>
+      <c r="I7" s="13" t="n"/>
+      <c r="J7" s="13" t="n"/>
+      <c r="K7" s="13" t="n"/>
+      <c r="L7" s="13" t="n"/>
+      <c r="M7" s="13" t="n"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>